<commit_message>
Insurgentes SD: EJE-B bottom 1#6 over the end wall
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mu9wxeehZ5MxBaqNG8frbT
</commit_message>
<xml_diff>
--- a/revit/ArmadoTrabes_Insurgentes/Armado_trabes_Nivel_Roof_Garden_N10.xlsx
+++ b/revit/ArmadoTrabes_Insurgentes/Armado_trabes_Nivel_Roof_Garden_N10.xlsx
@@ -5415,7 +5415,7 @@
       </c>
       <c r="S76" s="2" t="inlineStr">
         <is>
-          <t>Plano: bastones 2#6 sup. / 1#6 inf. de 100 cm dentro del muro (eje 8) a 120 cm del eje 8. Inf. 1#6 sobre el muro final (de 50 cm del eje 10 al extremo) no capturado. | secciones: T EJE-B Seccion 2 + T EJE-B Seccion 3 (se arman juntas; los bastones pasan el cambio de sección)</t>
+          <t>Plano: bastones 2#6 sup. / 1#6 inf. de 100 cm dentro del muro (eje 8) a 120 cm del eje 8. Inf. 1#6 sobre el muro final hasta el extremo: el botón lo arranca en el paño del muro (en el plano arranca 50 cm pasando el eje 10).</t>
         </is>
       </c>
     </row>
@@ -5533,7 +5533,11 @@
       <c r="J78" s="2" t="n"/>
       <c r="K78" s="2" t="n"/>
       <c r="L78" s="2" t="n"/>
-      <c r="M78" s="2" t="n"/>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>1#6 0</t>
+        </is>
+      </c>
       <c r="N78" s="2" t="n"/>
       <c r="O78" s="2" t="n"/>
       <c r="P78" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Insurgentes SD: Techos (N11) beams Excel; EJE-11 bar moved to support bastón
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mu9wxeehZ5MxBaqNG8frbT
</commit_message>
<xml_diff>
--- a/revit/ArmadoTrabes_Insurgentes/Armado_trabes_Nivel_Roof_Garden_N10.xlsx
+++ b/revit/ArmadoTrabes_Insurgentes/Armado_trabes_Nivel_Roof_Garden_N10.xlsx
@@ -4564,19 +4564,19 @@
         </is>
       </c>
       <c r="J63" s="2" t="n"/>
-      <c r="K63" s="2" t="n"/>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>2#8 280/60</t>
+        </is>
+      </c>
       <c r="L63" s="2" t="n"/>
-      <c r="M63" s="2" t="n"/>
-      <c r="N63" s="2" t="inlineStr">
-        <is>
-          <t>2#8 -100/-130</t>
-        </is>
-      </c>
-      <c r="O63" s="2" t="inlineStr">
-        <is>
-          <t>2#8 -100/-130</t>
-        </is>
-      </c>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>2#8 280/60</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="n"/>
+      <c r="O63" s="2" t="n"/>
       <c r="P63" s="2" t="inlineStr">
         <is>
           <t>E#3 @10</t>

</xml_diff>

<commit_message>
ArmadoVigasExcel: arm only some sections of a beam with [S1, S2]; split beams that are separate in the drawings
The button joined every touching section of a plan beam, but the drawings show some of them as separate
beams (T-5, T-6, EJE-5 on Roof Garden; EJE-3 on Techos). 'T-5 (viga 2) [S3]' now arms only those sections
as an independent beam; the Excel files use it where the drawing separates the pieces.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mu9wxeehZ5MxBaqNG8frbT
</commit_message>
<xml_diff>
--- a/revit/ArmadoTrabes_Insurgentes/Armado_trabes_Nivel_Roof_Garden_N10.xlsx
+++ b/revit/ArmadoTrabes_Insurgentes/Armado_trabes_Nivel_Roof_Garden_N10.xlsx
@@ -2339,7 +2339,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>EJE-5</t>
+          <t>EJE-5 [S1]</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="S29" s="2" t="inlineStr">
         <is>
-          <t>Plano: 15X80 con 3#8 y 15X60 con 3#4. Los tramos 4 y 5 (20x80, entre ejes L y K) no vienen detallados: se supuso 3#8 @10. | secciones: T EJE-5 Seccion 1 + T EJE-5 Seccion 2 (se arman juntas; los bastones pasan el cambio de sección)</t>
+          <t>En el plano son vigas separadas: 15X80 ejes N-L (S1, incluye la pieza de 20x80) y 15X60 ejes K-B (S2). | Plano: 15X80 con 3#8 y 15X60 con 3#4. Los tramos 4 y 5 (20x80, entre ejes L y K) no vienen detallados: se supuso 3#8 @10. | secciones: T EJE-5 Seccion 1 + T EJE-5 Seccion 2 (se arman juntas; los bastones pasan el cambio de sección)</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>EJE-5</t>
+          <t>EJE-5 [S1]</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -2465,7 +2465,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>EJE-5</t>
+          <t>EJE-5 [S1]</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -2534,7 +2534,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>EJE-5</t>
+          <t>EJE-5 [S1]</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>EJE-5</t>
+          <t>EJE-5 [S1]</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -2656,20 +2656,20 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>EJE-5</t>
+          <t>EJE-5 [S2]</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>5 (muro bajo la viga)</t>
+          <t>1 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>6 (muro)</t>
+          <t>2 (muro)</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -2707,7 +2707,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S34" s="2" t="n"/>
+      <c r="S34" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas: 15X80 ejes N-L (S1, incluye la pieza de 20x80) y 15X60 ejes K-B (S2).</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2717,20 +2721,20 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>EJE-5</t>
+          <t>EJE-5 [S2]</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>6 (muro)</t>
+          <t>2 (muro)</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>7 (muro bajo la viga)</t>
+          <t>3 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -2778,20 +2782,20 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>EJE-5</t>
+          <t>EJE-5 [S2]</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>7 (muro bajo la viga)</t>
+          <t>3 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>8 (muro bajo la viga)</t>
+          <t>4 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -2847,20 +2851,20 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>EJE-5</t>
+          <t>EJE-5 [S2]</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>8 (muro bajo la viga)</t>
+          <t>4 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>9 (muro bajo la viga)</t>
+          <t>5 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -2908,20 +2912,20 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>EJE-5</t>
+          <t>EJE-5 [S2]</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>9 (muro bajo la viga)</t>
+          <t>5 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>10 (muro bajo la viga)</t>
+          <t>6 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -2969,20 +2973,20 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>EJE-5</t>
+          <t>EJE-5 [S2]</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>10 (muro bajo la viga)</t>
+          <t>6 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>11 (muro bajo la viga)</t>
+          <t>7 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -11155,7 +11159,7 @@
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
-          <t>T-5 (viga 2)</t>
+          <t>T-5 (viga 2) [S1, S2]</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -11212,7 +11216,7 @@
       </c>
       <c r="S169" s="2" t="inlineStr">
         <is>
-          <t>Plano: ejes 5-8 (sup. 2#6, inf. 3#6, bastón sup. 3#6 del extremo a 120 cm pasando el muro) y ejes 9-11 (30X80, 3#12). Los tramos 5 y 6 (30x80 antes del eje 9) no vienen detallados: se supuso 3#12 @10. | secciones: T-5 Seccion 1 + T-5 Seccion 2 + T-5 Seccion 3 (se arman juntas; los bastones pasan el cambio de sección)</t>
+          <t>En el plano son vigas separadas: ejes 5-8 (S1+S2) y ejes 9-11 (S3, 30X80); cada parte se arma aparte. | Plano: ejes 5-8 (sup. 2#6, inf. 3#6, bastón sup. 3#6 del extremo a 120 cm pasando el muro) y ejes 9-11 (30X80, 3#12). Los tramos 5 y 6 (30x80 antes del eje 9) no vienen detallados: se supuso 3#12 @10. | secciones: T-5 Seccion 1 + T-5 Seccion 2 + T-5 Seccion 3 (se arman juntas; los bastones pasan el cambio de sección)</t>
         </is>
       </c>
     </row>
@@ -11224,7 +11228,7 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>T-5 (viga 2)</t>
+          <t>T-5 (viga 2) [S1, S2]</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -11285,7 +11289,7 @@
       </c>
       <c r="B171" s="2" t="inlineStr">
         <is>
-          <t>T-5 (viga 2)</t>
+          <t>T-5 (viga 2) [S1, S2]</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -11346,7 +11350,7 @@
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>T-5 (viga 2)</t>
+          <t>T-5 (viga 2) [S1, S2]</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -11407,15 +11411,15 @@
       </c>
       <c r="B173" s="2" t="inlineStr">
         <is>
-          <t>T-5 (viga 2)</t>
+          <t>T-5 (viga 2) [S3]</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D173" s="3" t="inlineStr">
         <is>
-          <t>5 (viga)</t>
+          <t>1 (viga)</t>
         </is>
       </c>
       <c r="E173" s="3" t="inlineStr">
@@ -11458,7 +11462,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S173" s="2" t="n"/>
+      <c r="S173" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas: ejes 5-8 (S1+S2) y ejes 9-11 (S3, 30X80); cada parte se arma aparte.</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -11468,11 +11476,11 @@
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>T-5 (viga 2)</t>
+          <t>T-5 (viga 2) [S3]</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D174" s="3" t="inlineStr">
         <is>
@@ -11481,7 +11489,7 @@
       </c>
       <c r="E174" s="3" t="inlineStr">
         <is>
-          <t>6 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="F174" t="n">
@@ -11529,20 +11537,20 @@
       </c>
       <c r="B175" s="2" t="inlineStr">
         <is>
-          <t>T-5 (viga 2)</t>
+          <t>T-5 (viga 2) [S3]</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D175" s="3" t="inlineStr">
         <is>
-          <t>6 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="E175" s="3" t="inlineStr">
         <is>
-          <t>7 (viga)</t>
+          <t>3 (viga)</t>
         </is>
       </c>
       <c r="F175" t="n">
@@ -11781,7 +11789,7 @@
       </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
-          <t>T-6 (viga 2)</t>
+          <t>T-6 (viga 2) [S2]</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -11838,7 +11846,7 @@
       </c>
       <c r="S179" s="2" t="inlineStr">
         <is>
-          <t>Los tramos 2 y 3 (30x80 entre ejes 8 y 9) no vienen detallados: se supuso @10. | secciones: T-6 Seccion 2 + T-6 Seccion 3 (se arman juntas; los bastones pasan el cambio de sección)</t>
+          <t>En el plano son vigas separadas: 30X80 (S2) y 15X80 (S3); cada parte se arma aparte. | Los tramos 2 y 3 (30x80 entre ejes 8 y 9) no vienen detallados: se supuso @10. | secciones: T-6 Seccion 2 + T-6 Seccion 3 (se arman juntas; los bastones pasan el cambio de sección)</t>
         </is>
       </c>
     </row>
@@ -11850,7 +11858,7 @@
       </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
-          <t>T-6 (viga 2)</t>
+          <t>T-6 (viga 2) [S2]</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -11911,7 +11919,7 @@
       </c>
       <c r="B181" s="2" t="inlineStr">
         <is>
-          <t>T-6 (viga 2)</t>
+          <t>T-6 (viga 2) [S2]</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -11972,20 +11980,20 @@
       </c>
       <c r="B182" s="2" t="inlineStr">
         <is>
-          <t>T-6 (viga 2)</t>
+          <t>T-6 (viga 2) [S3]</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D182" s="3" t="inlineStr">
         <is>
-          <t>3 (viga)</t>
+          <t>1 (viga)</t>
         </is>
       </c>
       <c r="E182" s="3" t="inlineStr">
         <is>
-          <t>4 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="F182" t="n">
@@ -12027,7 +12035,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S182" s="2" t="n"/>
+      <c r="S182" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas: 30X80 (S2) y 15X80 (S3); cada parte se arma aparte.</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
@@ -12037,20 +12049,20 @@
       </c>
       <c r="B183" s="2" t="inlineStr">
         <is>
-          <t>T-6 (viga 2)</t>
+          <t>T-6 (viga 2) [S3]</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D183" s="3" t="inlineStr">
         <is>
-          <t>4 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="E183" s="3" t="inlineStr">
         <is>
-          <t>5 (viga)</t>
+          <t>3 (viga)</t>
         </is>
       </c>
       <c r="F183" t="n">

</xml_diff>

<commit_message>
ArmadoVigasExcel: split a single-type beam by template spans ([T1-2]); split beams that are separate boxes in the drawings
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mu9wxeehZ5MxBaqNG8frbT
</commit_message>
<xml_diff>
--- a/revit/ArmadoTrabes_Insurgentes/Armado_trabes_Nivel_Roof_Garden_N10.xlsx
+++ b/revit/ArmadoTrabes_Insurgentes/Armado_trabes_Nivel_Roof_Garden_N10.xlsx
@@ -7370,7 +7370,7 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>EJE-J</t>
+          <t>EJE-J [T1-2]</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -7421,7 +7421,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S108" s="2" t="n"/>
+      <c r="S108" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas: ejes 3-8 (2#6) y ejes 8-10 (3#4); cada parte se arma aparte.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -7431,7 +7435,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>EJE-J</t>
+          <t>EJE-J [T1-2]</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -7492,20 +7496,20 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>EJE-J</t>
+          <t>EJE-J [T3]</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
-          <t>3 (viga)</t>
+          <t>1 (viga)</t>
         </is>
       </c>
       <c r="E110" s="3" t="inlineStr">
         <is>
-          <t>4 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="F110" t="n">
@@ -8923,7 +8927,7 @@
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>T-2 (viga 1)</t>
+          <t>T-2 (viga 1) [T1-2]</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -8976,7 +8980,7 @@
       </c>
       <c r="S133" s="2" t="inlineStr">
         <is>
-          <t>4 vigas separadas con esta trabe: cada una con sus filas (el paréntesis dice los ejes de sus extremos)</t>
+          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado. | 4 vigas separadas con esta trabe: cada una con sus filas (el paréntesis dice los ejes de sus extremos)</t>
         </is>
       </c>
     </row>
@@ -8988,7 +8992,7 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>T-2 (viga 1)</t>
+          <t>T-2 (viga 1) [T1-2]</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -9049,20 +9053,20 @@
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>T-2 (viga 1)</t>
+          <t>T-2 (viga 1) [T3]</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D135" s="3" t="inlineStr">
         <is>
-          <t>3 (viga)</t>
+          <t>1 (viga)</t>
         </is>
       </c>
       <c r="E135" s="3" t="inlineStr">
         <is>
-          <t>4 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="F135" t="n">
@@ -9100,7 +9104,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S135" s="2" t="n"/>
+      <c r="S135" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado.</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -9110,20 +9118,20 @@
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>T-2 (viga 1)</t>
+          <t>T-2 (viga 1) [T4-5]</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D136" s="3" t="inlineStr">
         <is>
-          <t>4 (viga)</t>
+          <t>1 (viga)</t>
         </is>
       </c>
       <c r="E136" s="3" t="inlineStr">
         <is>
-          <t>5 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="F136" t="n">
@@ -9161,7 +9169,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S136" s="2" t="n"/>
+      <c r="S136" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado.</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -9171,20 +9183,20 @@
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>T-2 (viga 1)</t>
+          <t>T-2 (viga 1) [T4-5]</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D137" s="3" t="inlineStr">
         <is>
-          <t>5 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="E137" s="3" t="inlineStr">
         <is>
-          <t>6 (viga)</t>
+          <t>3 (viga)</t>
         </is>
       </c>
       <c r="F137" t="n">
@@ -9232,7 +9244,7 @@
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>T-2 (viga 2)</t>
+          <t>T-2 (viga 2) [T1-2]</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -9283,7 +9295,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S138" s="2" t="n"/>
+      <c r="S138" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado.</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -9293,7 +9309,7 @@
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>T-2 (viga 2)</t>
+          <t>T-2 (viga 2) [T1-2]</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -9354,20 +9370,20 @@
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>T-2 (viga 2)</t>
+          <t>T-2 (viga 2) [T3]</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D140" s="3" t="inlineStr">
         <is>
-          <t>3 (viga)</t>
+          <t>1 (viga)</t>
         </is>
       </c>
       <c r="E140" s="3" t="inlineStr">
         <is>
-          <t>4 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="F140" t="n">
@@ -9405,7 +9421,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S140" s="2" t="n"/>
+      <c r="S140" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado.</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -9415,20 +9435,20 @@
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>T-2 (viga 2)</t>
+          <t>T-2 (viga 2) [T4-6]</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D141" s="3" t="inlineStr">
         <is>
-          <t>4 (viga)</t>
+          <t>1 (viga)</t>
         </is>
       </c>
       <c r="E141" s="3" t="inlineStr">
         <is>
-          <t>5 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="F141" t="n">
@@ -9466,7 +9486,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S141" s="2" t="n"/>
+      <c r="S141" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado.</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -9476,20 +9500,20 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>T-2 (viga 2)</t>
+          <t>T-2 (viga 2) [T4-6]</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D142" s="3" t="inlineStr">
         <is>
-          <t>5 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="E142" s="3" t="inlineStr">
         <is>
-          <t>6 (viga)</t>
+          <t>3 (viga)</t>
         </is>
       </c>
       <c r="F142" t="n">
@@ -9537,20 +9561,20 @@
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>T-2 (viga 2)</t>
+          <t>T-2 (viga 2) [T4-6]</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D143" s="3" t="inlineStr">
         <is>
-          <t>6 (viga)</t>
+          <t>3 (viga)</t>
         </is>
       </c>
       <c r="E143" s="3" t="inlineStr">
         <is>
-          <t>7 (viga)</t>
+          <t>4 (viga)</t>
         </is>
       </c>
       <c r="F143" t="n">
@@ -9842,7 +9866,7 @@
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>T-2' (viga 1)</t>
+          <t>T-2' (viga 1) [T1-2]</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -9895,7 +9919,7 @@
       </c>
       <c r="S148" s="2" t="inlineStr">
         <is>
-          <t>2 vigas separadas con esta trabe: cada una con sus filas (el paréntesis dice los ejes de sus extremos)</t>
+          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado. | 2 vigas separadas con esta trabe: cada una con sus filas (el paréntesis dice los ejes de sus extremos)</t>
         </is>
       </c>
     </row>
@@ -9907,7 +9931,7 @@
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>T-2' (viga 1)</t>
+          <t>T-2' (viga 1) [T1-2]</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -9968,20 +9992,20 @@
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>T-2' (viga 1)</t>
+          <t>T-2' (viga 1) [T3]</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D150" s="3" t="inlineStr">
         <is>
-          <t>3 (viga)</t>
+          <t>1 (viga)</t>
         </is>
       </c>
       <c r="E150" s="3" t="inlineStr">
         <is>
-          <t>4 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="F150" t="n">
@@ -10019,7 +10043,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S150" s="2" t="n"/>
+      <c r="S150" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado.</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -10029,20 +10057,20 @@
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>T-2' (viga 1)</t>
+          <t>T-2' (viga 1) [T4-5]</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D151" s="3" t="inlineStr">
         <is>
-          <t>4 (viga)</t>
+          <t>1 (viga)</t>
         </is>
       </c>
       <c r="E151" s="3" t="inlineStr">
         <is>
-          <t>5 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="F151" t="n">
@@ -10080,7 +10108,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S151" s="2" t="n"/>
+      <c r="S151" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado.</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -10090,20 +10122,20 @@
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>T-2' (viga 1)</t>
+          <t>T-2' (viga 1) [T4-5]</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D152" s="3" t="inlineStr">
         <is>
-          <t>5 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="E152" s="3" t="inlineStr">
         <is>
-          <t>6 (viga)</t>
+          <t>3 (viga)</t>
         </is>
       </c>
       <c r="F152" t="n">
@@ -11358,7 +11390,7 @@
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>T-6 (viga 1)</t>
+          <t>T-6 (viga 1) [T1]</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -11411,7 +11443,7 @@
       </c>
       <c r="S172" s="2" t="inlineStr">
         <is>
-          <t>2 vigas separadas con esta trabe: cada una con sus filas (el paréntesis dice los ejes de sus extremos)</t>
+          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado. | 2 vigas separadas con esta trabe: cada una con sus filas (el paréntesis dice los ejes de sus extremos)</t>
         </is>
       </c>
     </row>
@@ -11423,20 +11455,20 @@
       </c>
       <c r="B173" s="2" t="inlineStr">
         <is>
-          <t>T-6 (viga 1)</t>
+          <t>T-6 (viga 1) [T2]</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D173" s="3" t="inlineStr">
         <is>
+          <t>1 (viga)</t>
+        </is>
+      </c>
+      <c r="E173" s="3" t="inlineStr">
+        <is>
           <t>2 (viga)</t>
-        </is>
-      </c>
-      <c r="E173" s="3" t="inlineStr">
-        <is>
-          <t>3 (viga)</t>
         </is>
       </c>
       <c r="F173" t="n">
@@ -11474,7 +11506,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S173" s="2" t="n"/>
+      <c r="S173" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado.</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -11484,20 +11520,20 @@
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>T-6 (viga 1)</t>
+          <t>T-6 (viga 1) [T3]</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D174" s="3" t="inlineStr">
         <is>
-          <t>3 (viga)</t>
+          <t>1 (viga)</t>
         </is>
       </c>
       <c r="E174" s="3" t="inlineStr">
         <is>
-          <t>4 (muro)</t>
+          <t>2 (muro)</t>
         </is>
       </c>
       <c r="F174" t="n">
@@ -11535,7 +11571,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S174" s="2" t="n"/>
+      <c r="S174" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado.</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">

</xml_diff>